<commit_message>
Add country growth allocation runner
</commit_message>
<xml_diff>
--- a/data/coastal_datacenter_city_manifest.xlsx
+++ b/data/coastal_datacenter_city_manifest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\coastal_data_center\Code\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C434E35-A2ED-46C7-A73F-64F832BD55C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{121E7122-EEDF-4D6F-80B1-05C32DABB1CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="41180" windowHeight="21100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1316,17 +1316,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>median</t>
-  </si>
-  <si>
-    <t>upper_bound</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>lower_bound</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>total_gw_2030_Base</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -1340,6 +1329,18 @@
   </si>
   <si>
     <t>total_gw_2030_Headwinds</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>median_mw</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>upper_bound_mw</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>lower_bound_mw</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -1349,9 +1350,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
     <numFmt numFmtId="176" formatCode="000"/>
-    <numFmt numFmtId="182" formatCode="0_);[Red]\(0\)"/>
-    <numFmt numFmtId="183" formatCode="0.0_);[Red]\(0.0\)"/>
-    <numFmt numFmtId="186" formatCode="0.0000_);[Red]\(0.0000\)"/>
+    <numFmt numFmtId="177" formatCode="0_);[Red]\(0\)"/>
+    <numFmt numFmtId="178" formatCode="0.0_);[Red]\(0.0\)"/>
+    <numFmt numFmtId="179" formatCode="0.0000_);[Red]\(0.0000\)"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -1406,7 +1407,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -1432,21 +1433,24 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="182" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="182" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="186" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="183" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="182" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -6771,16 +6775,16 @@
         <v>419</v>
       </c>
       <c r="D1" s="9" t="s">
+        <v>427</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>428</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>429</v>
+      </c>
+      <c r="G1" s="9" t="s">
         <v>430</v>
-      </c>
-      <c r="E1" s="9" t="s">
-        <v>431</v>
-      </c>
-      <c r="F1" s="9" t="s">
-        <v>432</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>433</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -7155,14 +7159,14 @@
       <c r="C1" s="13" t="s">
         <v>426</v>
       </c>
-      <c r="D1" s="13" t="s">
-        <v>429</v>
-      </c>
-      <c r="E1" s="13" t="s">
-        <v>428</v>
-      </c>
-      <c r="F1" s="13" t="s">
-        <v>427</v>
+      <c r="D1" s="14" t="s">
+        <v>433</v>
+      </c>
+      <c r="E1" s="14" t="s">
+        <v>432</v>
+      </c>
+      <c r="F1" s="14" t="s">
+        <v>431</v>
       </c>
     </row>
     <row r="2" spans="1:6">

</xml_diff>